<commit_message>
content: sacred source workbooks + C-1c corrections (lap C-1d)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/source/hotico-content-en.xlsx
+++ b/content/source/hotico-content-en.xlsx
@@ -22,10 +22,13 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="264">
   <si>
+    <t>titlu video</t>
+  </si>
+  <si>
     <t>Denumire</t>
   </si>
   <si>
-    <t>titlu video</t>
+    <t>Areola reconstruction through dermopigmentation.</t>
   </si>
   <si>
     <t>descriere CTA (scris sub) Video</t>
@@ -34,49 +37,77 @@
     <t>Link youtube</t>
   </si>
   <si>
+    <t>link vimeo</t>
+  </si>
+  <si>
     <t>Eyebrow and Eyeliner Reconstruction in Cases of Alopecia</t>
   </si>
   <si>
-    <t>Areola reconstruction through dermopigmentation.</t>
+    <t>descriere text</t>
+  </si>
+  <si>
+    <t>link youtube</t>
+  </si>
+  <si>
+    <t>mini meniu de servicii</t>
   </si>
   <si>
     <t>Camouflaging scars through paramedical dermopigmentation</t>
   </si>
   <si>
-    <t>link vimeo</t>
-  </si>
-  <si>
-    <t>link youtube</t>
-  </si>
-  <si>
-    <t>descriere text</t>
-  </si>
-  <si>
-    <t>mini meniu de servicii</t>
-  </si>
-  <si>
     <t xml:space="preserve">cta sub titlu </t>
   </si>
   <si>
+    <t>Discover how caring for a finely drawn line can bring back your unique expression.</t>
+  </si>
+  <si>
+    <t>About HOTICO</t>
+  </si>
+  <si>
     <t>Discover how each carefully chosen shade can gently fade away the traces of the past.</t>
   </si>
   <si>
-    <t>Discover how caring for a finely drawn line can bring back your unique expression.</t>
+    <t>Discover how dermopigmentation art can gently close a painful chapter.</t>
+  </si>
+  <si>
+    <t>How can dermopigmentation bring natural beauty, emotional healing, and personal power? Discover the answer in this video manifesto by Alexandra Hotico.</t>
+  </si>
+  <si>
+    <t>Details</t>
   </si>
   <si>
     <t>cta intrebari</t>
   </si>
   <si>
+    <t>Am strâns cele mai importante întrebări și răspunsuri despre procedura dedicată alopeciei, ca să poți înțelege în detaliu cum redăm expresia naturală a feței. Dă click pe întrebare și lasă-mă să te ghidez pas cu pas prin video, dar și text.We have compiled the most important questions and answers about the alopecia procedure so that you can understand in detail how we restore the natural expression of the face. Click on the question and let me guide you step by step through the video and text.</t>
+  </si>
+  <si>
+    <t>We have compiled the most important questions and answers here to help you understand the procedure step by step. Click on the question and the video will take you directly to the complete explanation.</t>
+  </si>
+  <si>
+    <t>What is alopecia reconstruction through dermopigmentation?</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
     <t xml:space="preserve"> We have prepared the most important questions and answers about scar camouflage, explained clearly, both in text and video, so that you know exactly what to expect from this procedure.</t>
   </si>
   <si>
+    <t>What is areola reconstruction through dermopigmentation?</t>
+  </si>
+  <si>
     <t>What is scar camouflage through dermopigmentation?</t>
   </si>
   <si>
-    <t>About HOTICO</t>
-  </si>
-  <si>
-    <t>How can dermopigmentation bring natural beauty, emotional healing, and personal power? Discover the answer in this video manifesto by Alexandra Hotico.</t>
+    <t>https://youtu.be/sO2iJIfmV4A</t>
+  </si>
+  <si>
+    <t>There are moments in life when our bodies undergo profound changes, and our skin is left with scars that tell difficult stories. For many women, the loss of the areola after a mastectomy or other surgery is not only a physical change, but also an emotional one, which can affect how they see and feel about themselves.
+Reconstructive areola micropigmentation is a procedure that restores the natural appearance of the areola and nipple using advanced 3D micropigmentation techniques. Using a dermograph and pigments specially formulated to mimic the natural tones and shades of the skin, I create a realistic optical effect so that the areola appears three-dimensional, even when the tissue is flat.
+This procedure is especially recommended for women who have undergone mastectomy and breast reconstruction, but also for those who have discolored, asymmetrical, or altered areolas after surgery, breastfeeding, or trauma.
+In this type of dermopigmentation, technical precision is combined with artistic sensitivity and a deep respect for the privacy and story of each client. I choose the shades carefully, taking into account your skin tone and your wishes, so that the final result is as natural and harmonious as possible.
+The result is not only visible in the mirror, it is felt in the way you perceive yourself. For many women, this is the last step in the process of healing and reconnecting with their own body, a moment when they can look at themselves again with confidence and peace of mind.</t>
   </si>
   <si>
     <t>Every scar has a story. Some tell of healing, others of accidents or procedures that changed your life. But regardless of how they appeared: after surgery, an injury, an accident, a burn, or even from birth, as in the case of cleft lip, they can all bring back memories that you may not want to see every day in the mirror.
@@ -86,24 +117,6 @@
 The end result? More even-looking skin, where the scar becomes much less visible, and you can look at your body with more peace of mind and confidence.</t>
   </si>
   <si>
-    <t>https://youtu.be/sO2iJIfmV4A</t>
-  </si>
-  <si>
-    <t>https://youtu.be/ob1ZVybHtfw</t>
-  </si>
-  <si>
-    <t>Am strâns cele mai importante întrebări și răspunsuri despre procedura dedicată alopeciei, ca să poți înțelege în detaliu cum redăm expresia naturală a feței. Dă click pe întrebare și lasă-mă să te ghidez pas cu pas prin video, dar și text.We have compiled the most important questions and answers about the alopecia procedure so that you can understand in detail how we restore the natural expression of the face. Click on the question and let me guide you step by step through the video and text.</t>
-  </si>
-  <si>
-    <t>What is alopecia reconstruction through dermopigmentation?</t>
-  </si>
-  <si>
-    <t>Discover how dermopigmentation art can gently close a painful chapter.</t>
-  </si>
-  <si>
-    <t>Details</t>
-  </si>
-  <si>
     <t>When alopecia changes your appearance and takes away your eyebrows or eyelashes, you don't just lose hair, you lose part of your expression, part of how you recognize yourself in the mirror. For many people, this change brings insecurity, but also the desire to regain their familiar features.
 Paramedical dermopigmentation of the eyebrows and eyelash line is a specialized technique that restores the natural appearance of these areas using pigments and procedures adapted to hairless skin. Using a dermograph, I manually draw extremely fine hairs for the eyebrows, respecting the direction, thickness, and color of natural hairs, so that the result is realistic and harmonious.
 In the case of eyelashes, dermopigmentation is applied in the form of a lash enhancement: a very fine line at the base of the eyelashes, which creates the illusion of density and restores depth to the eyes, even when the eyelashes are completely missing.
@@ -111,16 +124,16 @@
 The end result is not just a face with eyebrows and a defined gaze, it is a step toward finding yourself again, regaining the expression that is so dear to you, and feeling like yourself once more.</t>
   </si>
   <si>
+    <t>https://youtu.be/Yhkyxca66tU</t>
+  </si>
+  <si>
     <t>https://youtu.be/TkoYLU4Q9Qs</t>
   </si>
   <si>
-    <t>We have compiled the most important questions and answers here to help you understand the procedure step by step. Click on the question and the video will take you directly to the complete explanation.</t>
-  </si>
-  <si>
-    <t>Price</t>
-  </si>
-  <si>
-    <t>What is areola reconstruction through dermopigmentation?</t>
+    <t>https://youtu.be/ob1ZVybHtfw</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711705/467b37802d?fl=ls&amp;fe=ec</t>
   </si>
   <si>
     <t>https://vimeo.com/1134711886/290ed60f4e?fl=ls&amp;fe=ec</t>
@@ -129,17 +142,19 @@
     <t>https://vimeo.com/1134714676/342cde51c4?fl=ls&amp;fe=ec</t>
   </si>
   <si>
-    <t>There are moments in life when our bodies undergo profound changes, and our skin is left with scars that tell difficult stories. For many women, the loss of the areola after a mastectomy or other surgery is not only a physical change, but also an emotional one, which can affect how they see and feel about themselves.
-Reconstructive areola micropigmentation is a procedure that restores the natural appearance of the areola and nipple using advanced 3D micropigmentation techniques. Using a dermograph and pigments specially formulated to mimic the natural tones and shades of the skin, I create a realistic optical effect so that the areola appears three-dimensional, even when the tissue is flat.
-This procedure is especially recommended for women who have undergone mastectomy and breast reconstruction, but also for those who have discolored, asymmetrical, or altered areolas after surgery, breastfeeding, or trauma.
-In this type of dermopigmentation, technical precision is combined with artistic sensitivity and a deep respect for the privacy and story of each client. I choose the shades carefully, taking into account your skin tone and your wishes, so that the final result is as natural and harmonious as possible.
-The result is not only visible in the mirror, it is felt in the way you perceive yourself. For many women, this is the last step in the process of healing and reconnecting with their own body, a moment when they can look at themselves again with confidence and peace of mind.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/Yhkyxca66tU</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711705/467b37802d?fl=ls&amp;fe=ec</t>
+    <t>https://vimeo.com/1134711759/a1599d08c3?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> What kind of pigments do I use?</t>
+  </si>
+  <si>
+    <t>When working with people who have alopecia, I know that choosing the right pigment is not just a matter of aesthetics, but also one of durability and safety. Skin affected by alopecia can react differently to pigment, depending on the cause of the condition, whether it is autoimmune, hormonal, hereditary, or related to medical treatments.
+For eyebrows, I choose hypoallergenic cosmetic pigments, free of heavy metals, specially formulated to remain stable and fade beautifully over time. I always adapt my selection to your skin undertone and any particularities caused by alopecia. If, for example, I know that your cellular metabolism is faster due to a medical condition, I choose pigments with a higher color concentration so that the result remains harmonious for as long as possible.
+For eyeliner, I use pigments with excellent stability, resistant to oxidation and color changes, because the eye area has thinner skin, but also because I want the line to remain clear and intense even after a few years.
+In both cases, the pigments are dermatologically tested, certified for cosmetic use, and selected to give you immediate beauty, but also the assurance that the result will remain clean, natural, and elegant in the long term, regardless of your type of alopecia.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Px2G7nEmgbw</t>
   </si>
   <si>
     <t>I'm the founder of HOTICO - Institut de Restauration. For over eight years I've worked in paramedical micropigmentation and permanent makeup, out of vocation.
@@ -150,19 +165,16 @@
 Here you find your beauty again. Here you come home.</t>
   </si>
   <si>
-    <t>https://vimeo.com/1134711759/a1599d08c3?fl=ls&amp;fe=ec</t>
+    <t>What kind of pigments do I use?</t>
+  </si>
+  <si>
+    <t>Gallery</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711731/c84c2f313d?fl=ls&amp;fe=ec</t>
   </si>
   <si>
     <t>How HOTICO works</t>
-  </si>
-  <si>
-    <t>Discover how each procedure begins with you, your story, and a personalized, safe, and empathetic process.</t>
-  </si>
-  <si>
-    <t>What kind of pigments do I use?</t>
-  </si>
-  <si>
-    <t>https://youtu.be/ngoI9KMIckw</t>
   </si>
   <si>
     <t>When working on scars, it is a matter of covering an area, but also of integrating it perfectly into the rest of the skin so that it no longer attracts attention. This means that the pigment must be chosen with extreme precision, both in terms of shade and formula.
@@ -171,31 +183,13 @@
 The color's resistance can also be influenced by the texture of the scar; more fibrous areas may retain the pigment differently, which is why I adjust the concentration and implantation technique. All these details are part of a careful process, in which my goal is to create visual harmony that restores your self-confidence.</t>
   </si>
   <si>
+    <t>Discover how each procedure begins with you, your story, and a personalized, safe, and empathetic process.</t>
+  </si>
+  <si>
     <t>https://youtu.be/7HnFLAR3VVc</t>
   </si>
   <si>
-    <t xml:space="preserve"> What kind of pigments do I use?</t>
-  </si>
-  <si>
-    <t>When working with people who have alopecia, I know that choosing the right pigment is not just a matter of aesthetics, but also one of durability and safety. Skin affected by alopecia can react differently to pigment, depending on the cause of the condition, whether it is autoimmune, hormonal, hereditary, or related to medical treatments.
-For eyebrows, I choose hypoallergenic cosmetic pigments, free of heavy metals, specially formulated to remain stable and fade beautifully over time. I always adapt my selection to your skin undertone and any particularities caused by alopecia. If, for example, I know that your cellular metabolism is faster due to a medical condition, I choose pigments with a higher color concentration so that the result remains harmonious for as long as possible.
-For eyeliner, I use pigments with excellent stability, resistant to oxidation and color changes, because the eye area has thinner skin, but also because I want the line to remain clear and intense even after a few years.
-In both cases, the pigments are dermatologically tested, certified for cosmetic use, and selected to give you immediate beauty, but also the assurance that the result will remain clean, natural, and elegant in the long term, regardless of your type of alopecia.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/Px2G7nEmgbw</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134714635/1860dc6d53?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>Gallery</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711905/d3be87eaf6?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711731/c84c2f313d?fl=ls&amp;fe=ec</t>
+    <t>https://youtu.be/ngoI9KMIckw</t>
   </si>
   <si>
     <t xml:space="preserve">"What kind of pigments do I use for reconstructive areola micropigmentation?"
@@ -224,6 +218,39 @@
 In short: it is not completely sensation-free, but it is a procedure designed to be gentle, safe, and bearable, so that your experience is as relaxed and stress-free as possible.</t>
   </si>
   <si>
+    <t>https://youtu.be/kqk8FgxrJ5M</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134714613/53378a3329?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711905/d3be87eaf6?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134714635/1860dc6d53?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711764/6cf21b660f?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Can I do this while breastfeeding?</t>
+  </si>
+  <si>
+    <t>This is one of the questions I get asked most often, and I want to give you a sincere and complete answer. In theory, cosmetic dermopigmentation only acts on the superficial layers of the skin, using biocompatible pigments and local anesthetics applied to the surface. I work with sterile, single-use consumables in an environment that complies with all hygiene and safety standards.
+However, according to best practice recommendations, all aesthetic procedures, including dermopigmentation, are contraindicated during pregnancy and breastfeeding. The reason? The precautionary principle. Even if the risk of adverse reactions is low, the body undergoes significant hormonal and physiological changes, and any additional stress or local reaction can influence your general condition and, indirectly, breastfeeding.
+My recommendation, as a professional, is to postpone the procedure until after breastfeeding or at least until the last few months, when breastfeeding is no longer exclusive. It is the safest choice for both you and your baby.
+Your safety and health always come first. Dermopigmentation is about beauty, but above all about care, responsibility, and respect for your body.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/0NxmDb_DaDo</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134714593/f808dbf7db?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>"What you need to do before alopecia dermopigmentation"</t>
+  </si>
+  <si>
     <t>Everything starts with you and your story. At the initial consultation I listen and I understand what you want. Every result is built on your features, your skin tone, your medical history and your pace.
 I use pigments formulated specifically for cosmetic and paramedical micropigmentation, medically safe and tested for stability over time. I choose the shades so they blend naturally into the skin.
 The equipment is the latest generation, all materials are sterile and single-use, and hygiene protocols follow the guidelines of the Swiss Federal Office of Public Health (FOPH) and the EU REACH regulation.
@@ -231,34 +258,60 @@
 When you settle onto my treatment table, you breathe and leave the rest to me. You're in good hands, from the choice of pigment to the last line drawn.</t>
   </si>
   <si>
-    <t>https://youtu.be/kqk8FgxrJ5M</t>
-  </si>
-  <si>
     <t>Learn with HOTICO</t>
   </si>
   <si>
-    <t>https://vimeo.com/1134711764/6cf21b660f?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
     <t>Find out why paramedical dermopigmentation is the future of your profession and how dedicated training can change your career path.</t>
   </si>
   <si>
     <t>https://youtu.be/Ru5ZCOs_d9o</t>
   </si>
   <si>
-    <t>https://vimeo.com/1134714613/53378a3329?fl=ls&amp;fe=ec</t>
+    <t xml:space="preserve">
+Alopecia—whether patchy, total, or caused by medical factors and treatments such as chemotherapy brings with it not only aesthetic but also practical challenges. When eyebrows and eyelashes are missing, dermopigmentation can restore facial harmony, expressiveness, and confidence. But before we get there, proper preparation is essential for a beautiful and stable result.
+First, we need to know the cause of the alopecia. If it is autoimmune or hormonal in nature (alopecia areata, thyroiditis, menopause), the skin in the area may be more sensitive or have a different ability to fix the pigment. If hair loss was caused by cancer treatments, it is essential to wait at least 6 months after their completion and to have the approval of the attending physician. In the case of alopecia without an active medical cause, the procedure can be performed as soon as the skin is healthy.
+Skin hydration is crucial, without hair, the skin of the eyebrows and eyelids tends to be more exposed to wind, sun, or cold, which can dry it out quickly. In the weeks leading up to the procedure, use a gentle, fragrance-free cream to maintain skin elasticity.
+Avoid aggressive procedures in the eye and eyebrow area at least 2 weeks before: waxing, acid treatments, microdermabrasion, or chemical peels. These can irritate the skin and affect how the pigment sets.
+On the day of the procedure, avoid coffee, alcohol, and aspirin or ibuprofen, all of which can increase sensitivity and the risk of bleeding. If you wear contact lenses, bring a sterile case to store them in during the eyeliner procedure.
+In the case of alopecia, a very important detail is the personalized design. We don't just draw a "beautiful" eyebrow shape and a "visually pleasing" eyeliner, we work to reconstruct the natural expression of your face, taking into account symmetry, proportions, and features. For this reason, on the day of your appointment, I will do a complete simulation on your skin so that you can see and approve the result before we start dermopigmentation.
+If I notice that your skin is irritated, extremely dry, or that there is local inflammation, we will reschedule. This is not a postponement, but a professional choice to ensure that the result is uniform, stable, and truly beautiful.
+Preparation before eyebrow and eyeliner dermopigmentation in cases of alopecia is essentially a combination of physical care and medical clarity. And I am here to ensure that when you arrive at my work bed, both your skin and you, as a person, are ready for a transformation that will restore the harmony and expressiveness of your gaze.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/GAbv0id7-iA</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711721/6aa7761199?fl=ls&amp;fe=ec</t>
   </si>
   <si>
     <t>https://vimeo.com/1134714690/ce241187c3?fl=ls&amp;fe=ec</t>
   </si>
   <si>
-    <t xml:space="preserve"> Can I do this while breastfeeding?</t>
-  </si>
-  <si>
-    <t>This is one of the questions I get asked most often, and I want to give you a sincere and complete answer. In theory, cosmetic dermopigmentation only acts on the superficial layers of the skin, using biocompatible pigments and local anesthetics applied to the surface. I work with sterile, single-use consumables in an environment that complies with all hygiene and safety standards.
-However, according to best practice recommendations, all aesthetic procedures, including dermopigmentation, are contraindicated during pregnancy and breastfeeding. The reason? The precautionary principle. Even if the risk of adverse reactions is low, the body undergoes significant hormonal and physiological changes, and any additional stress or local reaction can influence your general condition and, indirectly, breastfeeding.
-My recommendation, as a professional, is to postpone the procedure until after breastfeeding or at least until the last few months, when breastfeeding is no longer exclusive. It is the safest choice for both you and your baby.
-Your safety and health always come first. Dermopigmentation is about beauty, but above all about care, responsibility, and respect for your body.</t>
+    <t>What happens immediately after and how do I maintain the procedure?</t>
+  </si>
+  <si>
+    <t>In the first few hours, your eyebrows or eyeliner will appear more intense and darker in color. This is completely normal, as the pigment is still on the surface and your skin is responding to the procedure. During this phase, I will show you exactly how to gently clean the area so that you can remove excess lymph without disturbing the skin. It is very important not to touch the area with dirty hands and to completely avoid direct moisture or exposure to heat and steam. Swimming pools, saunas, and hot showers are not an option during the first week.
+As the skin begins to regenerate, small scabs may appear. I know the temptation to peel them off can be great, but please let them fall off on their own. If you remove them prematurely, you risk removing the pigment from the skin, leaving areas without color that can only be corrected with a touch-up. I will recommend a special healing balm, which you should apply in a very thin layer, with clean hands or a cosmetic stick, several times a day.
+In the case of eyeliner, it is normal to feel slight sensitivity or notice a little swelling of the eyelids. A simple cold compress, applied several times a day, helps enormously to soothe the area. It is equally important to avoid makeup around the eyes, mascara, or oily makeup removers until the skin is completely healed.
+Sunscreen is another step you can't skip. Even in winter, UV rays can damage pigment, so I recommend either applying SPF to your eyebrows daily after healing or wearing large sunglasses with UV protection for your eyeliner.
+You should also know that when working with alopecia, the skin can react differently depending on the cause of the condition, whether it is an autoimmune disease, cancer treatment, or a hormonal imbalance. Sometimes the pigment takes perfectly the first time, other times we need a more careful touch-up to fix it evenly. That's why I like to keep in touch with you during the healing period and see you for a check-up to make sure we get the best possible result.
+In short, I bring my expertise and attention to detail, you bring your care for yourself in the first few weeks, and together we make your eyebrows or eyeliner exactly as you wanted them, beautiful, natural, and long-lasting.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Z8ooi5NcfAw</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711696/d2a7485551?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>Why are two procedures necessary?</t>
+  </si>
+  <si>
+    <t>This is a question I get asked very often, and it's natural for you to have it in mind too. The short answer is: because every skin is unique and reacts differently to pigment.
+After the first dermopigmentation session, the treated area, whether it's the eyebrows, lips, or areolas. looks more intense. The pigment has just been deposited, and the skin is slightly inflamed. Over the next few weeks, during the natural healing process, the color begins to fade and settle until it reaches its final shade.
+During this period, the skin naturally eliminates a percentage of the pigment. This is the body's normal reaction to any element introduced from outside. This is where retouching comes in: it is the second session in which we fill in the areas where the pigment has settled less, even out the color, adjust the symmetry if necessary, and strengthen the contours.
+Retouching is essential for a uniform, long-lasting, and natural-looking result. Once the skin has "gotten used" to the pigment during the first procedure, it will accept it much better during the second, which makes the final result stable and beautiful over time.
+In short: the first procedure prepares the ground, and the touch-up completes the job. Without touch-ups, the result is only half done. With touch-ups, you get the eyebrows, lips, or areolas you want, for longer and without surprises.</t>
   </si>
   <si>
     <t>The years spent working with women after a mastectomy, surgery or an accident taught me that a precise hand changes the way someone sees herself.
@@ -267,31 +320,22 @@
 I'll pass on safe protocols, techniques adapted to every skin type, and the right way to speak to a vulnerable patient. You finish the training confident with scar camouflage and areola tattooing. Your patients feel it from the first session, and their trust becomes your capital.</t>
   </si>
   <si>
+    <t>https://youtu.be/3hGfw3MSc4A</t>
+  </si>
+  <si>
+    <t>What is Paramedical Dermopigmentation?</t>
+  </si>
+  <si>
     <t>Can I do this while breastfeeding?</t>
   </si>
   <si>
-    <t>https://youtu.be/0NxmDb_DaDo</t>
-  </si>
-  <si>
-    <t>What is Paramedical Dermopigmentation?</t>
-  </si>
-  <si>
     <t>Discover step by step where paramedical dermopigmentation is applied and why it has such a huge emotional impact.</t>
   </si>
   <si>
-    <t>https://youtu.be/xWkn9WosGz0</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134714593/f808dbf7db?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134714662/4f2609f849?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
     <t>"What you need to do before areola dermopigmentation"</t>
   </si>
   <si>
-    <t>"What you need to do before alopecia dermopigmentation"</t>
+    <t>https://vimeo.com/1134714625/d065d5d624?fl=ls&amp;fe=ec</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -308,34 +352,40 @@
     <t>https://youtu.be/vX6ZBGQAi2g</t>
   </si>
   <si>
+    <t>How long does the pigment last?</t>
+  </si>
+  <si>
+    <t>When it comes to dermopigmentation of eyebrows or eyelashes lost due to alopecia, durability can vary from person to person. On average, for eyebrows we are talking about 1 to 3 years, and for eyeliner, i.e. the pigment line on the eyelids, 2 to 4 years, because the eye area is more protected and less exposed to factors that degrade the pigment.
+The difference depends on the cause of alopecia. If we are talking about areata alopecia, an autoimmune condition that affects only the hair follicles but leaves the skin healthy, the durability may be similar to that of a person who does not have alopecia. On the other hand, if alopecia is related to thyroid problems, hormonal disorders, certain nutritional deficiencies, or if it appeared after cancer treatments, the skin may retain pigment for less time, precisely because of changes in the body.
+There are also rarer situations, such as scarring alopecia, where the skin is fibrotic, and there the results can be more unpredictable.
+That is why, before the procedure, I like to discuss the medical history in detail and adapt the technique, pigment, and work plan so that we achieve the best possible result for each individual case. Ultimately, it is important that the procedure is performed at the right time, on prepared and healthy skin, so that you can enjoy beautiful, defined eyebrows or eyelashes for as long as possible.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Lc7Xvh2IZ1U</t>
+  </si>
+  <si>
+    <t>https://youtu.be/xWkn9WosGz0</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711743/5bdc0c91b3?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711785/f2f2bbd1f6?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>in formularul de programare la pasul 2 - sub alege data</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134714662/4f2609f849?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>Would you like another procedure?</t>
+  </si>
+  <si>
     <t>What you need to do before scar camouflage?</t>
   </si>
   <si>
-    <t>Paramedical micropigmentation restores the appearance of the skin after trauma, surgery or a medical condition, using advanced pigments and techniques.
-You'll find it in areola tattooing after a mastectomy, in scar camouflage, in evening out the skin tone of stable vitiligo, and in brow and lash restoration where hair has been lost. Cosmetic tattooing brings your features forward. Paramedical micropigmentation gives you back your identity.
-Pigment sits in the surface layer of the skin and blends naturally with your skin tone, with no harsh colour, no visible edges. The result is long-lasting and fades gradually, so we can adjust it as your skin or your needs change.
-I work with the latest generation of equipment, medical-grade pigments and sterile, single-use materials, following strict hygiene protocols. Every piece of work is adapted to your skin and to your story.
-You look in the mirror and you recognise yourself. It's the start of a chapter where your body and your story move forward, on your terms.</t>
-  </si>
-  <si>
-    <t>What is Cosmetic Dermopigmentation?</t>
-  </si>
-  <si>
-    <t>Discover how cosmetic dermopigmentation enhances your natural beauty discreetly and harmoniously, without the tattoo effect.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Alopecia—whether patchy, total, or caused by medical factors and treatments such as chemotherapy brings with it not only aesthetic but also practical challenges. When eyebrows and eyelashes are missing, dermopigmentation can restore facial harmony, expressiveness, and confidence. But before we get there, proper preparation is essential for a beautiful and stable result.
-First, we need to know the cause of the alopecia. If it is autoimmune or hormonal in nature (alopecia areata, thyroiditis, menopause), the skin in the area may be more sensitive or have a different ability to fix the pigment. If hair loss was caused by cancer treatments, it is essential to wait at least 6 months after their completion and to have the approval of the attending physician. In the case of alopecia without an active medical cause, the procedure can be performed as soon as the skin is healthy.
-Skin hydration is crucial, without hair, the skin of the eyebrows and eyelids tends to be more exposed to wind, sun, or cold, which can dry it out quickly. In the weeks leading up to the procedure, use a gentle, fragrance-free cream to maintain skin elasticity.
-Avoid aggressive procedures in the eye and eyebrow area at least 2 weeks before: waxing, acid treatments, microdermabrasion, or chemical peels. These can irritate the skin and affect how the pigment sets.
-On the day of the procedure, avoid coffee, alcohol, and aspirin or ibuprofen, all of which can increase sensitivity and the risk of bleeding. If you wear contact lenses, bring a sterile case to store them in during the eyeliner procedure.
-In the case of alopecia, a very important detail is the personalized design. We don't just draw a "beautiful" eyebrow shape and a "visually pleasing" eyeliner, we work to reconstruct the natural expression of your face, taking into account symmetry, proportions, and features. For this reason, on the day of your appointment, I will do a complete simulation on your skin so that you can see and approve the result before we start dermopigmentation.
-If I notice that your skin is irritated, extremely dry, or that there is local inflammation, we will reschedule. This is not a postponement, but a professional choice to ensure that the result is uniform, stable, and truly beautiful.
-Preparation before eyebrow and eyeliner dermopigmentation in cases of alopecia is essentially a combination of physical care and medical clarity. And I am here to ensure that when you arrive at my work bed, both your skin and you, as a person, are ready for a transformation that will restore the harmony and expressiveness of your gaze.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/dOcTKS42t8Y</t>
+    <t xml:space="preserve"> What happens immediately after and how do I maintain the procedure?</t>
   </si>
   <si>
     <t>Scar camouflage is one of those procedures that not only changes the appearance of your skin, but also the way you see and feel yourself in your own body. Whether we are talking about post-operative scars, scars from an accident, a burn, or even lip reconstruction following a cleft lip, proper preparation before the procedure is the key to a beautiful and natural result.
@@ -348,35 +398,7 @@
 Preparing for scar camouflage is not complicated, but every detail matters enormously. I bring my experience and trained eye, you bring your prepared skin, and together we make that scar go unnoticed, and you see yourself as whole again.</t>
   </si>
   <si>
-    <t>https://youtu.be/GAbv0id7-iA</t>
-  </si>
-  <si>
     <t>https://youtu.be/YDGsGaQboUQ</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711785/f2f2bbd1f6?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134714645/1ec654d870?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711721/6aa7761199?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711942/35d581cfb3?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> What happens immediately after and how do I maintain the procedure?</t>
-  </si>
-  <si>
-    <t>Cosmetic tattooing is a delicate procedure. I place pigment into the surface layer of the skin to bring your features into balance. You'll also hear it called permanent makeup or semi-permanent makeup, and it's most often done on the brows, lips and eyeliner.
-Pigment stays near the surface and fades gradually, so you stay free to change the result. It's formulated specifically for the face, works with your skin tone and gives a natural finish.
-The technique brings out your natural beauty. It redefines the brow shape, brightens and evens the lips, and softly defines the lash line.
-I work with the latest generation of equipment and medical-grade pigments, chosen to suit your skin tone. Results last between 1 and 3 years depending on your skin type, then we schedule a touch-up.
-You gain time every morning. You wake up with your face already done, you look in the mirror and see yourself rested, exactly you, just a little more defined.</t>
-  </si>
-  <si>
-    <t>sub logo si poza -&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -392,10 +414,36 @@
     <t>https://youtu.be/Cj3-EfPse04</t>
   </si>
   <si>
-    <t>What happens immediately after and how do I maintain the procedure?</t>
-  </si>
-  <si>
-    <t>The art that heals</t>
+    <t>Paramedical micropigmentation restores the appearance of the skin after trauma, surgery or a medical condition, using advanced pigments and techniques.
+You'll find it in areola tattooing after a mastectomy, in scar camouflage, in evening out the skin tone of stable vitiligo, and in brow and lash restoration where hair has been lost. Cosmetic tattooing brings your features forward. Paramedical micropigmentation gives you back your identity.
+Pigment sits in the surface layer of the skin and blends naturally with your skin tone, with no harsh colour, no visible edges. The result is long-lasting and fades gradually, so we can adjust it as your skin or your needs change.
+I work with the latest generation of equipment, medical-grade pigments and sterile, single-use materials, following strict hygiene protocols. Every piece of work is adapted to your skin and to your story.
+You look in the mirror and you recognise yourself. It's the start of a chapter where your body and your story move forward, on your terms.</t>
+  </si>
+  <si>
+    <t>What is Cosmetic Dermopigmentation?</t>
+  </si>
+  <si>
+    <t>Discover how cosmetic dermopigmentation enhances your natural beauty discreetly and harmoniously, without the tattoo effect.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/dOcTKS42t8Y</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711774/de054ab2bf?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711942/35d581cfb3?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134714645/1ec654d870?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>This is a question I get asked very often, and it's natural for you to have it in mind too. The short answer is: because every skin is unique and reacts differently to pigment.
+After the first dermopigmentation session, the treated area, whether it's the eyebrows, lips, or areolas, looks more intense. The pigment has just been deposited, and the skin is slightly inflamed. Over the next few weeks, during the natural healing process, the color begins to fade and settle until it reaches its final shade.
+During this period, the skin naturally eliminates a percentage of the pigment. This is the body's normal reaction to any element introduced from outside. This is where retouching comes in: it is the second session in which we fill in the areas where the pigment has settled less, even out the color, adjust the symmetry if necessary, and strengthen the contours.
+Retouching is essential for a uniform, long-lasting, and natural-looking result. Once the skin has "gotten used" to the pigment during the first procedure, it will accept it much better during the second, which makes the final result stable and beautiful over time.
+In short: the first procedure prepares the ground, and the touch-up completes the job. Without touch-ups, the result is only half done. With touch-ups, you get the eyebrows, lips, or areolas you want, for longer and without surprises.</t>
   </si>
   <si>
     <t>After we camouflage a scar, an equally important stage begins: the healing period. The skin we have worked on has already undergone a regeneration process in the past, and now it needs a little more patience and attention for the pigment to set nicely and evenly.
@@ -409,20 +457,25 @@
     <t>https://youtu.be/8I84vJi_c5s</t>
   </si>
   <si>
-    <t>In the first few hours, your eyebrows or eyeliner will appear more intense and darker in color. This is completely normal, as the pigment is still on the surface and your skin is responding to the procedure. During this phase, I will show you exactly how to gently clean the area so that you can remove excess lymph without disturbing the skin. It is very important not to touch the area with dirty hands and to completely avoid direct moisture or exposure to heat and steam. Swimming pools, saunas, and hot showers are not an option during the first week.
-As the skin begins to regenerate, small scabs may appear. I know the temptation to peel them off can be great, but please let them fall off on their own. If you remove them prematurely, you risk removing the pigment from the skin, leaving areas without color that can only be corrected with a touch-up. I will recommend a special healing balm, which you should apply in a very thin layer, with clean hands or a cosmetic stick, several times a day.
-In the case of eyeliner, it is normal to feel slight sensitivity or notice a little swelling of the eyelids. A simple cold compress, applied several times a day, helps enormously to soothe the area. It is equally important to avoid makeup around the eyes, mascara, or oily makeup removers until the skin is completely healed.
-Sunscreen is another step you can't skip. Even in winter, UV rays can damage pigment, so I recommend either applying SPF to your eyebrows daily after healing or wearing large sunglasses with UV protection for your eyeliner.
-You should also know that when working with alopecia, the skin can react differently depending on the cause of the condition, whether it is an autoimmune disease, cancer treatment, or a hormonal imbalance. Sometimes the pigment takes perfectly the first time, other times we need a more careful touch-up to fix it evenly. That's why I like to keep in touch with you during the healing period and see you for a check-up to make sure we get the best possible result.
-In short, I bring my expertise and attention to detail, you bring your care for yourself in the first few weeks, and together we make your eyebrows or eyeliner exactly as you wanted them, beautiful, natural, and long-lasting.</t>
+    <t>Cosmetic tattooing is a delicate procedure. I place pigment into the surface layer of the skin to bring your features into balance. You'll also hear it called permanent makeup or semi-permanent makeup, and it's most often done on the brows, lips and eyeliner.
+Pigment stays near the surface and fades gradually, so you stay free to change the result. It's formulated specifically for the face, works with your skin tone and gives a natural finish.
+The technique brings out your natural beauty. It redefines the brow shape, brightens and evens the lips, and softly defines the lash line.
+I work with the latest generation of equipment and medical-grade pigments, chosen to suit your skin tone. Results last between 1 and 3 years depending on your skin type, then we schedule a touch-up.
+You gain time every morning. You wake up with your face already done, you look in the mirror and see yourself rested, exactly you, just a little more defined.</t>
+  </si>
+  <si>
+    <t>sub logo si poza -&gt;</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711925/940adaa1c1?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>The art that heals</t>
   </si>
   <si>
     <t>An institute where beauty and healing naturally intertwine: cosmetic dermopigmentation for naturalness, paramedical dermopigmentation for emotional balance, and advanced training for those who want to become artists of empathy and transformation.</t>
   </si>
   <si>
-    <t>https://youtu.be/Z8ooi5NcfAw</t>
-  </si>
-  <si>
     <t>deasupra de video -&gt; CTA</t>
   </si>
   <si>
@@ -436,9 +489,6 @@
   </si>
   <si>
     <t>The steps of your transformation</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711774/de054ab2bf?fl=ls&amp;fe=ec</t>
   </si>
   <si>
     <t>Consulting</t>
@@ -454,12 +504,17 @@
 </t>
   </si>
   <si>
-    <t>https://vimeo.com/1134711925/940adaa1c1?fl=ls&amp;fe=ec</t>
+    <t>Areola micropigmentation is, by its nature and purpose, a procedure designed to last. We use organic pigments specially designed for areola reconstruction, chosen precisely for their stability over time. The result? A beautiful, harmonious color that retains its vitality for years, without visible or unpleasant changes.
+Unlike other areas of the body, the areola is not constantly exposed to the sun or factors that can accelerate pigment fading, which contributes to its almost permanent resistance. Thus, a single procedure performed correctly, followed by the initial touch-up, can bring a long-lasting result that does not require frequent refreshments.
+This is also why reconstructive dermopigmentation of the areola is considered a final, stable, and safe step in the breast reconstruction process—a procedure that offers peace of mind, safety, and a body image with which you can feel at peace again, day after day, year after year.</t>
   </si>
   <si>
     <t>Procedure</t>
   </si>
   <si>
+    <t>https://youtu.be/7E1Dy2Dq4kI</t>
+  </si>
+  <si>
     <t>1. Personalized analysis and preparation. We sit down, discuss your expectations and desires, and I analyze your skin and the area to be treated, taking into account your medical history, skin type, and undertone. Then we draw the ideal shape together, analyze it visually, and adjust it until we both feel it is perfect for you. We choose the right shade, a pigment that will blend naturally with your skin.</t>
   </si>
   <si>
@@ -469,18 +524,25 @@
     <t>3. Completion and post-procedure care. After completing the procedure, we analyze the result and explain step by step how to care for the pigmented area during the healing period. Depending on your skin type and the procedure, you will receive personalized recommendations for maintenance so that the result remains natural, stable, and beautiful over time.</t>
   </si>
   <si>
+    <t>This is a question I get asked very often, and it's natural for you to have it in mind too. The short answer is: because every skin is unique and reacts differently to pigment.
+After the first dermopigmentation session, the treated area—whether it's the eyebrows, lips, or areolas—looks more intense. The pigment has just been deposited, and the skin is slightly inflamed. Over the next few weeks, during the natural healing process, the color begins to fade and settle until it reaches its final shade.
+During this period, the skin naturally eliminates a percentage of the pigment. This is the body's normal reaction to any element introduced from the outside. This is where retouching comes in: it is the second session in which we fill in the areas where the pigment has settled less, even out the color, adjust the symmetry if necessary, and strengthen the contours.
+Touch-ups are essential for a uniform, long-lasting, and natural-looking result. Once the skin has "gotten used" to the pigment during the first procedure, it will accept it much better during the second, which makes the final result stable and beautiful over time.
+In short: the first procedure prepares the ground, and the touch-up finishes the job. Without touch-ups, the result is only half complete. With touch-ups, you get the eyebrows, lips, or areolas you want, for longer and without surprises.</t>
+  </si>
+  <si>
     <t>Touch-up</t>
   </si>
   <si>
     <t>1. Post-healing analysis. After 4-6 weeks, when the skin is completely healed, we meet again to perform the touch-up. We analyze together how the pigment has settled and discuss any adjustments: shape, shade, or final intensity. At this stage, you play an active role because, after observing how the color has gradually changed during healing, you can now clearly express your preferences regarding the desired final intensity.</t>
   </si>
   <si>
-    <t>https://vimeo.com/1134711696/d2a7485551?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
     <t>2. Retouching. This is the consolidation stage, in which we intervene again on the area, applying pigment where necessary for uniformity and stability. The procedure is the same as the first session, but without redrawing the shape, we are already working with a beautiful, agreed base, which we are perfecting. The goal is to fix the color and provide a uniform, natural, and durable result.</t>
   </si>
   <si>
+    <t>https://vimeo.com/1134711800/365f64eb51?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
     <t>3. Color refreshment. After a few years, depending on skin type and procedure, I recommend a maintenance session. At this stage, the color is gently refreshed to maintain a fresh and harmonious appearance. We do not redraw or reconstruct, we only revitalize the pigment so that the result remains natural and elegant over time.</t>
   </si>
   <si>
@@ -491,6 +553,15 @@
   </si>
   <si>
     <t>Bifa GDPR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imagine that we are giving the skin the chance to blend in harmoniously; that is essentially what we do when we camouflage scars. On average, the result can last between 3 and 5 years, sometimes even longer, if your skin is well cared for and protected.
+Durability depends greatly on a few key elements: your skin type, the pigment used, sun exposure, and, of course, how you care for the area after the procedure. Moisturized skin, protected with SPF and without harsh products, will keep the pigment vibrant for a long time.
+Like any work of finesse, scar camouflage comes with a little secret: it is normal to need periodic touch-ups. Not because something is wrong, but because the skin changes its tone slightly over time (yes, even the most stable pigment lightens a little), and everyday life exposes us to sun, chemicals, or normal wear and tear. So a maintenance session is what helps us keep the perfect shade.
+</t>
+  </si>
+  <si>
+    <t>https://youtu.be/IyLn8I5lDds</t>
   </si>
   <si>
     <r>
@@ -528,86 +599,15 @@
     </r>
   </si>
   <si>
-    <t>Why are two procedures necessary?</t>
+    <t>https://vimeo.com/1134711965/98c5f6fdd6?fl=ls&amp;fe=ec</t>
   </si>
   <si>
     <t xml:space="preserve">buton Next </t>
   </si>
   <si>
-    <t>This is a question I get asked very often, and it's natural for you to have it in mind too. The short answer is: because every skin is unique and reacts differently to pigment.
-After the first dermopigmentation session, the treated area, whether it's the eyebrows, lips, or areolas, looks more intense. The pigment has just been deposited, and the skin is slightly inflamed. Over the next few weeks, during the natural healing process, the color begins to fade and settle until it reaches its final shade.
-During this period, the skin naturally eliminates a percentage of the pigment. This is the body's normal reaction to any element introduced from outside. This is where retouching comes in: it is the second session in which we fill in the areas where the pigment has settled less, even out the color, adjust the symmetry if necessary, and strengthen the contours.
-Retouching is essential for a uniform, long-lasting, and natural-looking result. Once the skin has "gotten used" to the pigment during the first procedure, it will accept it much better during the second, which makes the final result stable and beautiful over time.
-In short: the first procedure prepares the ground, and the touch-up completes the job. Without touch-ups, the result is only half done. With touch-ups, you get the eyebrows, lips, or areolas you want, for longer and without surprises.</t>
-  </si>
-  <si>
     <t>Reviews</t>
   </si>
   <si>
-    <t>https://youtu.be/3hGfw3MSc4A</t>
-  </si>
-  <si>
-    <t>This is a question I get asked very often, and it's natural for you to have it in mind too. The short answer is: because every skin is unique and reacts differently to pigment.
-After the first dermopigmentation session, the treated area—whether it's the eyebrows, lips, or areolas—looks more intense. The pigment has just been deposited, and the skin is slightly inflamed. Over the next few weeks, during the natural healing process, the color begins to fade and settle until it reaches its final shade.
-During this period, the skin naturally eliminates a percentage of the pigment. This is the body's normal reaction to any element introduced from the outside. This is where retouching comes in: it is the second session in which we fill in the areas where the pigment has settled less, even out the color, adjust the symmetry if necessary, and strengthen the contours.
-Touch-ups are essential for a uniform, long-lasting, and natural-looking result. Once the skin has "gotten used" to the pigment during the first procedure, it will accept it much better during the second, which makes the final result stable and beautiful over time.
-In short: the first procedure prepares the ground, and the touch-up finishes the job. Without touch-ups, the result is only half complete. With touch-ups, you get the eyebrows, lips, or areolas you want, for longer and without surprises.</t>
-  </si>
-  <si>
-    <t>This is a question I get asked very often, and it's natural for you to have it in mind too. The short answer is: because every skin is unique and reacts differently to pigment.
-After the first dermopigmentation session, the treated area, whether it's the eyebrows, lips, or areolas. looks more intense. The pigment has just been deposited, and the skin is slightly inflamed. Over the next few weeks, during the natural healing process, the color begins to fade and settle until it reaches its final shade.
-During this period, the skin naturally eliminates a percentage of the pigment. This is the body's normal reaction to any element introduced from outside. This is where retouching comes in: it is the second session in which we fill in the areas where the pigment has settled less, even out the color, adjust the symmetry if necessary, and strengthen the contours.
-Retouching is essential for a uniform, long-lasting, and natural-looking result. Once the skin has "gotten used" to the pigment during the first procedure, it will accept it much better during the second, which makes the final result stable and beautiful over time.
-In short: the first procedure prepares the ground, and the touch-up completes the job. Without touch-ups, the result is only half done. With touch-ups, you get the eyebrows, lips, or areolas you want, for longer and without surprises.</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134714625/d065d5d624?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>How long does the pigment last?</t>
-  </si>
-  <si>
-    <t>Areola micropigmentation is, by its nature and purpose, a procedure designed to last. We use organic pigments specially designed for areola reconstruction, chosen precisely for their stability over time. The result? A beautiful, harmonious color that retains its vitality for years, without visible or unpleasant changes.
-Unlike other areas of the body, the areola is not constantly exposed to the sun or factors that can accelerate pigment fading, which contributes to its almost permanent resistance. Thus, a single procedure performed correctly, followed by the initial touch-up, can bring a long-lasting result that does not require frequent refreshments.
-This is also why reconstructive dermopigmentation of the areola is considered a final, stable, and safe step in the breast reconstruction process—a procedure that offers peace of mind, safety, and a body image with which you can feel at peace again, day after day, year after year.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/7E1Dy2Dq4kI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imagine that we are giving the skin the chance to blend in harmoniously; that is essentially what we do when we camouflage scars. On average, the result can last between 3 and 5 years, sometimes even longer, if your skin is well cared for and protected.
-Durability depends greatly on a few key elements: your skin type, the pigment used, sun exposure, and, of course, how you care for the area after the procedure. Moisturized skin, protected with SPF and without harsh products, will keep the pigment vibrant for a long time.
-Like any work of finesse, scar camouflage comes with a little secret: it is normal to need periodic touch-ups. Not because something is wrong, but because the skin changes its tone slightly over time (yes, even the most stable pigment lightens a little), and everyday life exposes us to sun, chemicals, or normal wear and tear. So a maintenance session is what helps us keep the perfect shade.
-</t>
-  </si>
-  <si>
-    <t>https://youtu.be/IyLn8I5lDds</t>
-  </si>
-  <si>
-    <t>When it comes to dermopigmentation of eyebrows or eyelashes lost due to alopecia, durability can vary from person to person. On average, for eyebrows we are talking about 1 to 3 years, and for eyeliner, i.e. the pigment line on the eyelids, 2 to 4 years, because the eye area is more protected and less exposed to factors that degrade the pigment.
-The difference depends on the cause of alopecia. If we are talking about areata alopecia, an autoimmune condition that affects only the hair follicles but leaves the skin healthy, the durability may be similar to that of a person who does not have alopecia. On the other hand, if alopecia is related to thyroid problems, hormonal disorders, certain nutritional deficiencies, or if it appeared after cancer treatments, the skin may retain pigment for less time, precisely because of changes in the body.
-There are also rarer situations, such as scarring alopecia, where the skin is fibrotic, and there the results can be more unpredictable.
-That is why, before the procedure, I like to discuss the medical history in detail and adapt the technique, pigment, and work plan so that we achieve the best possible result for each individual case. Ultimately, it is important that the procedure is performed at the right time, on prepared and healthy skin, so that you can enjoy beautiful, defined eyebrows or eyelashes for as long as possible.</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711800/365f64eb51?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>https://youtu.be/Lc7Xvh2IZ1U</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711965/98c5f6fdd6?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711743/5bdc0c91b3?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>in formularul de programare la pasul 2 - sub alege data</t>
-  </si>
-  <si>
-    <t>Would you like another procedure?</t>
-  </si>
-  <si>
     <t>pasul 3</t>
   </si>
   <si>
@@ -620,6 +620,9 @@
     <t>ce se intampla daca bifeaza DA</t>
   </si>
   <si>
+    <t>decriere raspuns din video</t>
+  </si>
+  <si>
     <t>Have you undergone a mastectomy or other breast surgery?</t>
   </si>
   <si>
@@ -635,22 +638,42 @@
     <t>-&gt;consultatie online whatsapp + lista de asteptare</t>
   </si>
   <si>
+    <t>Eyebrows redefined through hair stroke technique dermopigmentation</t>
+  </si>
+  <si>
     <t>Did you experience any complications after the procedure (infection, delayed healing, necrosis, radiodermatitis)?</t>
   </si>
   <si>
+    <t>Discover how a delicate procedure brings symmetry and naturalness to your eyebrows.</t>
+  </si>
+  <si>
     <t>Did you undergo radiation therapy in the chest area?</t>
   </si>
   <si>
     <t>daca bifeaza trebuie sa apara alte 2 optiuni</t>
   </si>
   <si>
+    <t>Here you will find the explanations you need to understand how eyebrow dermopigmentation works and what results you can achieve. We have answered all your questions so that you can understand the process and feel confident.</t>
+  </si>
+  <si>
     <t>Column 2: Have you developed fibrosis? Yes/No</t>
   </si>
   <si>
+    <t>What is brows dermopigmentation?</t>
+  </si>
+  <si>
     <t>Did you undergo chemotherapy?</t>
   </si>
   <si>
-    <t>decriere raspuns din video</t>
+    <t>Eyebrows are one of the most important features of the face. They define your expression, frame your eyes, and can completely change the harmony of your face. Eyebrow dermopigmentation is a method that allows us to restore the shape, density, and aesthetic balance of your eyebrows, using colors that are naturally adapted to your skin and features.
+Instead of resorting to makeup or pencil every day, this technique uses fine, controlled pigmentation to achieve a long-lasting result that looks as natural as possible.
+One of my favorite methods is the hair-by-hair technique performed with a dermograph. Instead of covering the area with a block of color, I manually draw extremely fine lines with the help of a professional dermopigmentation device, which perfectly mimic natural hairs. Each "hair" is drawn individually, respecting the direction, thickness, and length of your real hairs, and the pigment is carefully chosen to match the shade of your eyebrows and skin.
+The dermograph gives me very precise control over the depth and fineness of each hair, which means that the result looks realistic both up close and from a distance. The procedure is completely personalized so that the final shape perfectly matches your physiognomy, expression, and lifestyle.
+Because the pigment is introduced superficially, it fades beautifully over time, allowing for adjustments when your preferences or facial features change.
+The end result? Symmetrical, natural-looking eyebrows that enhance your eyes and give you the freedom to wake up every morning looking well-groomed, without makeup and without effort.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/8-XL9WYzoA8</t>
   </si>
   <si>
     <t>Has your skin developed? 
@@ -671,50 +694,30 @@
     <t>Do you have the approval of your oncologist or surgeon for the dermopigmentation procedure?</t>
   </si>
   <si>
-    <t>Eyebrows redefined through hair stroke technique dermopigmentation</t>
-  </si>
-  <si>
     <t>daca bifeaza da -&gt; programare, dar aici ar trebui sa apara automat bifa cu DA sau NU in cazul in care la prima intrebare (cea legata de mastectomie fiindca sunt femei care au avut marire sau micsorare si atunci nu se incadreaza la acordul medicului oncolog) a bifat DA</t>
   </si>
   <si>
-    <t>Discover how a delicate procedure brings symmetry and naturalness to your eyebrows.</t>
-  </si>
-  <si>
     <t>Does your skin tend to form hypertrophic scars or keloids?</t>
   </si>
   <si>
     <t>-&gt;consultatie online whatsapp</t>
   </si>
   <si>
-    <t>Here you will find the explanations you need to understand how eyebrow dermopigmentation works and what results you can achieve. We have answered all your questions so that you can understand the process and feel confident.</t>
-  </si>
-  <si>
-    <t>What is brows dermopigmentation?</t>
-  </si>
-  <si>
     <t>Are there any hardened, very fibrous, or irradiated areas (very stiff skin) in the treatment area?</t>
   </si>
   <si>
     <t>Do you have any autoimmune diseases (e.g., lupus, Hashimoto's disease, vitiligo, psoriasis)?</t>
   </si>
   <si>
-    <t>Eyebrows are one of the most important features of the face. They define your expression, frame your eyes, and can completely change the harmony of your face. Eyebrow dermopigmentation is a method that allows us to restore the shape, density, and aesthetic balance of your eyebrows, using colors that are naturally adapted to your skin and features.
-Instead of resorting to makeup or pencil every day, this technique uses fine, controlled pigmentation to achieve a long-lasting result that looks as natural as possible.
-One of my favorite methods is the hair-by-hair technique performed with a dermograph. Instead of covering the area with a block of color, I manually draw extremely fine lines with the help of a professional dermopigmentation device, which perfectly mimic natural hairs. Each "hair" is drawn individually, respecting the direction, thickness, and length of your real hairs, and the pigment is carefully chosen to match the shade of your eyebrows and skin.
-The dermograph gives me very precise control over the depth and fineness of each hair, which means that the result looks realistic both up close and from a distance. The procedure is completely personalized so that the final shape perfectly matches your physiognomy, expression, and lifestyle.
-Because the pigment is introduced superficially, it fades beautifully over time, allowing for adjustments when your preferences or facial features change.
-The end result? Symmetrical, natural-looking eyebrows that enhance your eyes and give you the freedom to wake up every morning looking well-groomed, without makeup and without effort.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/8-XL9WYzoA8</t>
-  </si>
-  <si>
     <t>Do you have a weakened immune system or are you undergoing treatment with immunosuppressants?</t>
   </si>
   <si>
     <t>Are you undergoing treatment with corticosteroids (pills, injections, or creams applied to the affected area)?</t>
   </si>
   <si>
+    <t>https://vimeo.com/1134712951/e107454150?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
     <t>Are you currently taking antibiotics?</t>
   </si>
   <si>
@@ -733,16 +736,10 @@
     <t>Have you recently had any treatments in the chest area (laser, peels, microneedling, PRP)?</t>
   </si>
   <si>
+    <t>Microblading vs Hair stroke dermopigmentation?</t>
+  </si>
+  <si>
     <t>Have you had corticosteroid injections in your scars?</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134712951/e107454150?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>If you are unsure, write us a few words about your situation and we will do a personalized online assessment.</t>
-  </si>
-  <si>
-    <t>Microblading vs Hair stroke dermopigmentation?</t>
   </si>
   <si>
     <t>Microblading vs. hair-by-hair. This is a question I get asked very often, and it's important to understand the differences because they affect not only the appearance of your eyebrows but also the long-term health of your skin.
@@ -753,6 +750,9 @@
 In short: microblading cuts the skin and offers shorter-lasting and riskier results, while hair-by-hair dermopigmentation with a dermograph respects the skin, heals faster, lasts longer, and offers a flawless natural look. It is the choice I confidently recommend for beautiful, healthy, and harmonious eyebrows in the long term.</t>
   </si>
   <si>
+    <t>If you are unsure, write us a few words about your situation and we will do a personalized online assessment.</t>
+  </si>
+  <si>
     <t>https://youtu.be/Yo3jhzJLu-g</t>
   </si>
   <si>
@@ -769,34 +769,6 @@
   </si>
   <si>
     <t>https://vimeo.com/1134712983/56498a90c2?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>descriere raspuns</t>
-  </si>
-  <si>
-    <t>Defined look with eyeliner dermopigmentation</t>
-  </si>
-  <si>
-    <t>Discover how eyeliner dermopigmentation can add depth to your gaze with everyday elegance.</t>
-  </si>
-  <si>
-    <t>Your questions are natural. My answers are here to guide you and show you how safe and gentle the procedure is.</t>
-  </si>
-  <si>
-    <t>What is eyeliner dermopigmentation?</t>
-  </si>
-  <si>
-    <t>The eyes always tell a story, and the fine line at the base of the eyelashes can subtly change the expression of the eyes and the way you perceive yourself in the mirror. Eyeliner dermopigmentation is a technique I use to highlight and define the lash line, creating more expressive and brighter eyes without the need for daily makeup.
-It is an ideal choice if you want to save time in the morning, no longer worry about eyeliner smudging or fading throughout the day, or if you have sensitive eyes and want to avoid applying cosmetics daily.
-The procedure is performed with a professional dermograph and special pigments, which are very finely applied at the base of the eyelashes. Depending on your preferences, the line can be extremely discreet, just to accentuate the eyes, or slightly more pronounced, for an effect similar to perfectly applied makeup.
-Eyeliner dermopigmentation does not weigh down the eyes, does not create an artificial look, and is customized according to the shape of the eyes, the color of the iris, and your lifestyle. The result can last between 2 and 5 years, fading naturally over time, and the intensity can be refreshed whenever you want.
-The end result? A fine, harmonious, and expressive contour that brightens your eyes and gives you the confidence that your eyes look flawless at any time of the day, effortlessly.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/e42uuKwrjAs</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134712009/e0cd18d47e?fl=ls&amp;fe=ec</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -813,6 +785,81 @@
   </si>
   <si>
     <t xml:space="preserve">
+This is one of the questions I get asked most often, and I want to give you a sincere and complete answer. In theory, cosmetic dermopigmentation only acts on the superficial layers of the skin, using biocompatible pigments and local anesthetics applied to the surface. I work with sterile, single-use consumables in an environment that complies with all hygiene and safety standards.
+However, according to best practice recommendations, all aesthetic procedures, including dermopigmentation, are contraindicated during pregnancy and breastfeeding. The reason? The precautionary principle. Even if the risk of adverse reactions is low, the body undergoes significant hormonal and physiological changes, and any additional stress or local reaction can influence your general condition and, indirectly, breastfeeding.
+My recommendation, as a professional, is to postpone the procedure until after breastfeeding or at least until the last few months, when breastfeeding is no longer exclusive. It is the safest choice for both you and your baby.
+Your safety and health always come first. Dermopigmentation is about beauty, but above all about care, responsibility, and respect for your body.</t>
+  </si>
+  <si>
+    <t>What you need to do before brows dermopigmentation?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Before we start working on your eyebrows, we want to make sure that the area is in the best possible condition. A beautiful result always starts with healthy, well-prepared skin.
+A few days before the procedure, make sure you drink enough water and keep the skin around your eyebrows well hydrated. If you have dry skin, use a gentle cream or moisturizing serum, but avoid products with retinol, acids (AHA/BHA), or vitamin C in the eyebrow area, as they can sensitize the skin. And if you have oily skin, it's best to avoid excess sebum on the day of the procedure: gentle cleansing in the morning will suffice.
+Very important: at least 48 hours before, avoid tanning beds, prolonged sun exposure, or aggressive treatments on the eyebrow area (waxing, chemical peels, microdermabrasion). All of these can irritate the skin and affect its ability to retain pigment.
+On the day of your appointment, do not consume coffee, green tea, energy drinks, alcohol, or blood-thinning medications (aspirin, anti-inflammatories, omega-3 supplements, ginkgo biloba) without informing me in advance. All of these can increase sensitivity and cause slight bleeding during the procedure, which affects pigment retention.
+If you have extremely sensitive skin or are prone to redness, I will guide you in making small adjustments to your skincare routine to reduce the risk of irritation. And if you are undergoing medical treatment or have a dermatological condition in the eyebrow area, we will discuss together to determine the ideal time for the procedure.
+One more thing: if you come in with your natural eyebrow shape, without any drastic tweezing in the last few weeks, you give me more freedom to create a harmonious shape that is tailored exactly to your features.
+In short, the preparation is simple, but it matters a lot: you come with care for yourself, I come with experience and perfect technique, and together we make your eyebrows exactly how you want them: beautiful, natural, and long-lasting.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/zw1e2Mz9dCA</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134712955/75508ccb8b?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>descriere raspuns</t>
+  </si>
+  <si>
+    <t>Defined look with eyeliner dermopigmentation</t>
+  </si>
+  <si>
+    <t>After eyebrow dermopigmentation, how you care for them in the first few days is absolutely essential for how beautifully and evenly the pigment will set. The first 7-10 days are the period when the skin heals, and what you do or don't do now can make the difference between a flawless result and one with small gaps in color.
+In the first few hours after the procedure, your eyebrows will look more intense and darker in color, which is normal, as the pigment is still on the surface. I will explain exactly how to gently clean the area so that you remove excess lymph without disturbing the skin. It is very important not to touch them with dirty hands and not to wet them directly. Hot showers, steam, swimming pools, or saunas are prohibited during the first week.
+As the healing process begins, small scabs will form. This is where one of the biggest mistakes you can make comes in: picking at them. Do not touch them, do not scratch them, let them fall off on their own. If you remove them prematurely, you risk removing the pigment from the skin, leaving gaps that can only be repaired with touch-ups. I will recommend a special healing balm, which you should apply in a very thin layer, only with clean hands or a cosmetic stick, several times a day.
+Once the scabs have fallen off completely, we can say that we are entering the second stage of care. The skin is still sensitive, so we continue to avoid exfoliating products, AHA/BHA acids, retinol, or vitamin C in the eyebrow area for at least a month. And if you want the result to remain beautiful in the long term, sun protection is mandatory — SPF 30 or even 50, applied daily to the eyebrows, whether it's summer or winter.
+Keep in mind: we always evaluate the final result after touch-ups, not after the first session. In the first few weeks, the color will go through several stages — it will fade, even out, and only then will it reveal its true beauty. I am here to guide you step by step, I will provide you with a personalized care guide, and if you follow all these instructions, your eyebrows will look flawless and enhance your face for a long time.</t>
+  </si>
+  <si>
+    <t>Discover how eyeliner dermopigmentation can add depth to your gaze with everyday elegance.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/qpF18FTEhR0</t>
+  </si>
+  <si>
+    <t>Your questions are natural. My answers are here to guide you and show you how safe and gentle the procedure is.</t>
+  </si>
+  <si>
+    <t>What is eyeliner dermopigmentation?</t>
+  </si>
+  <si>
+    <t>The eyes always tell a story, and the fine line at the base of the eyelashes can subtly change the expression of the eyes and the way you perceive yourself in the mirror. Eyeliner dermopigmentation is a technique I use to highlight and define the lash line, creating more expressive and brighter eyes without the need for daily makeup.
+It is an ideal choice if you want to save time in the morning, no longer worry about eyeliner smudging or fading throughout the day, or if you have sensitive eyes and want to avoid applying cosmetics daily.
+The procedure is performed with a professional dermograph and special pigments, which are very finely applied at the base of the eyelashes. Depending on your preferences, the line can be extremely discreet, just to accentuate the eyes, or slightly more pronounced, for an effect similar to perfectly applied makeup.
+Eyeliner dermopigmentation does not weigh down the eyes, does not create an artificial look, and is customized according to the shape of the eyes, the color of the iris, and your lifestyle. The result can last between 2 and 5 years, fading naturally over time, and the intensity can be refreshed whenever you want.
+The end result? A fine, harmonious, and expressive contour that brightens your eyes and gives you the confidence that your eyes look flawless at any time of the day, effortlessly.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/e42uuKwrjAs</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134712943/777ba19052?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134712009/e0cd18d47e?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+This is a question I get asked very often, and it's natural for you to have it in mind too. The short answer is: because every skin is unique and reacts differently to pigment.
+After the first dermopigmentation session, the treated area, whether it's the eyebrows, lips, or areolas, looks more intense. The pigment is freshly deposited, and the skin is slightly inflamed. Over the next few weeks, during the natural healing process, the color begins to fade and settle until it reaches its final shade.
+During this period, the skin naturally eliminates a percentage of the pigment. This is the body's normal reaction to any element introduced from the outside. This is where the touch-up comes in: it is the second session in which we fill in the areas where the pigment has settled less, even out the color, adjust the symmetry if necessary, and strengthen the contours.
+Touch-ups are essential for a uniform, long-lasting, and natural-looking result. Once the skin has "gotten used" to the pigment during the first procedure, it will accept it much better during the second, which makes the final result stable and beautiful over time.
+In short: the first procedure prepares the ground, and the touch-up finishes the job. Without touch-ups, the result is only half complete. With touch-ups, you get the eyebrows, lips, or areolas you want, for longer and without surprises.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
 For me, eyeliner is not just a line drawn on the eyelid. It is that detail that changes the entire expression of your gaze and that must remain beautiful and clear for years. And it all starts with the pigment.
 I only work with premium cosmetic pigments, created specifically for the sensitive eye area, biocompatible and hypoallergenic. This means that the skin accepts them easily, without irritation and without the risk of the color changing to blue, green, or gray over time. I always choose pure shades with a stable formula so that the line retains its intensity without fading unsightly.
 Before choosing the final pigment, I analyze your skin tone, eye color, and the effect you want: whether you want an intense, cat-eye look or a more discreet and natural effect. The pigment is not just "black or brown"; it is specially tailored to you so that the eyeliner enhances your beauty, not detracts from it.
@@ -822,42 +869,20 @@
     <t>https://youtu.be/68nVeP9YPx0</t>
   </si>
   <si>
-    <t xml:space="preserve">
-This is one of the questions I get asked most often, and I want to give you a sincere and complete answer. In theory, cosmetic dermopigmentation only acts on the superficial layers of the skin, using biocompatible pigments and local anesthetics applied to the surface. I work with sterile, single-use consumables in an environment that complies with all hygiene and safety standards.
-However, according to best practice recommendations, all aesthetic procedures, including dermopigmentation, are contraindicated during pregnancy and breastfeeding. The reason? The precautionary principle. Even if the risk of adverse reactions is low, the body undergoes significant hormonal and physiological changes, and any additional stress or local reaction can influence your general condition and, indirectly, breastfeeding.
-My recommendation, as a professional, is to postpone the procedure until after breastfeeding or at least until the last few months, when breastfeeding is no longer exclusive. It is the safest choice for both you and your baby.
-Your safety and health always come first. Dermopigmentation is about beauty, but above all about care, responsibility, and respect for your body.</t>
+    <t>The duration of the results varies, but in general, you can enjoy beautiful eyebrows for between 1 and 3 years. The difference depends on several factors: skin type, the shade of pigment chosen, lifestyle, and, above all, aftercare.
+In the first few weeks, the eyebrows go through a natural healing process: the color gradually lightens and settles evenly. To preserve the result for as long as possible, it is important to let the skin heal at its own pace, not to remove the scabs, and to protect the area from the sun by always using a high SPF.
+In the long term, there are factors that can accelerate pigment fading, such as products containing vitamin C, retinoids, or exfoliating acids, frequent exposure to chlorinated water, or tanning beds. Lighter shades, such as blonde or light brown, also tend to lose their intensity faster than darker ones.
+To maintain a clear shape and vibrant color, I recommend maintenance touch-ups whenever you feel your eyebrows need a refresh.
+Essentially, I lay the foundation for a lasting result, and you, through daily care, keep it beautiful for as long as possible.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Lq8mWDiICOg</t>
   </si>
   <si>
     <t>https://vimeo.com/1134714017/c5473672e3?fl=ls&amp;fe=ec</t>
   </si>
   <si>
-    <t>link raspuns</t>
-  </si>
-  <si>
-    <t>Defined smile through lips dermopigmentation</t>
-  </si>
-  <si>
-    <t>Discover how lip dermopigmentation can add depth and sensuality to your smile.</t>
-  </si>
-  <si>
-    <t>We have prepared the most important questions and answers about lip dermopigmentation, explained clearly, both in text and video, so that you know exactly what to expect from this procedure.</t>
-  </si>
-  <si>
-    <t>What is lips dermopigmentation?</t>
-  </si>
-  <si>
-    <t>A smile is one of the most beautiful expressions we wear, and the color and contour of the lips can give it more harmony and radiance. Lip dermopigmentation is a technique by which I delicately restore or intensify the natural shade of the lips, correct small asymmetries, and create a fine contour, so that they always look full of life.
-It is an ideal choice if your lips are very pale, have lost pigment over time, or if you want to even out the color or give them a fresher and more defined look without using lipstick every day.
-The procedure is performed using a professional dermograph and special pigments, chosen in shades that match your skin tone and complement your features. The final result can be very discreet, for a natural "my lips but better" effect, or more intense, depending on your wishes.
-Lip dermopigmentation does not mean a strong, rigid color, but a transparent, warm shade that blends perfectly with the texture of your lips. The pigment gradually fades over time, allowing you to adjust or refresh the color whenever you feel the need.
-The end result? Lips with a more defined contour, uniform color, and healthy appearance that will make your smile stand out in the most beautiful way, every day, effortlessly.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/5mVL5l7AcaQ</t>
-  </si>
-  <si>
-    <t>What you need to do before brows dermopigmentation?</t>
+    <t>https://vimeo.com/1134712991/2a713496a8?fl=ls&amp;fe=ec</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -873,30 +898,29 @@
 In short: it is not completely sensation-free, but it is a procedure designed to be gentle, safe, and bearable, so that your experience is as relaxed and stress-free as possible.</t>
   </si>
   <si>
-    <t xml:space="preserve">
-Before we start working on your eyebrows, we want to make sure that the area is in the best possible condition. A beautiful result always starts with healthy, well-prepared skin.
-A few days before the procedure, make sure you drink enough water and keep the skin around your eyebrows well hydrated. If you have dry skin, use a gentle cream or moisturizing serum, but avoid products with retinol, acids (AHA/BHA), or vitamin C in the eyebrow area, as they can sensitize the skin. And if you have oily skin, it's best to avoid excess sebum on the day of the procedure: gentle cleansing in the morning will suffice.
-Very important: at least 48 hours before, avoid tanning beds, prolonged sun exposure, or aggressive treatments on the eyebrow area (waxing, chemical peels, microdermabrasion). All of these can irritate the skin and affect its ability to retain pigment.
-On the day of your appointment, do not consume coffee, green tea, energy drinks, alcohol, or blood-thinning medications (aspirin, anti-inflammatories, omega-3 supplements, ginkgo biloba) without informing me in advance. All of these can increase sensitivity and cause slight bleeding during the procedure, which affects pigment retention.
-If you have extremely sensitive skin or are prone to redness, I will guide you in making small adjustments to your skincare routine to reduce the risk of irritation. And if you are undergoing medical treatment or have a dermatological condition in the eyebrow area, we will discuss together to determine the ideal time for the procedure.
-One more thing: if you come in with your natural eyebrow shape, without any drastic tweezing in the last few weeks, you give me more freedom to create a harmonious shape that is tailored exactly to your features.
-In short, the preparation is simple, but it matters a lot: you come with care for yourself, I come with experience and perfect technique, and together we make your eyebrows exactly how you want them: beautiful, natural, and long-lasting.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/zw1e2Mz9dCA</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711822/0140c6e130?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134712955/75508ccb8b?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>After eyebrow dermopigmentation, how you care for them in the first few days is absolutely essential for how beautifully and evenly the pigment will set. The first 7-10 days are the period when the skin heals, and what you do or don't do now can make the difference between a flawless result and one with small gaps in color.
-In the first few hours after the procedure, your eyebrows will look more intense and darker in color, which is normal, as the pigment is still on the surface. I will explain exactly how to gently clean the area so that you remove excess lymph without disturbing the skin. It is very important not to touch them with dirty hands and not to wet them directly. Hot showers, steam, swimming pools, or saunas are prohibited during the first week.
-As the healing process begins, small scabs will form. This is where one of the biggest mistakes you can make comes in: picking at them. Do not touch them, do not scratch them, let them fall off on their own. If you remove them prematurely, you risk removing the pigment from the skin, leaving gaps that can only be repaired with touch-ups. I will recommend a special healing balm, which you should apply in a very thin layer, only with clean hands or a cosmetic stick, several times a day.
-Once the scabs have fallen off completely, we can say that we are entering the second stage of care. The skin is still sensitive, so we continue to avoid exfoliating products, AHA/BHA acids, retinol, or vitamin C in the eyebrow area for at least a month. And if you want the result to remain beautiful in the long term, sun protection is mandatory — SPF 30 or even 50, applied daily to the eyebrows, whether it's summer or winter.
-Keep in mind: we always evaluate the final result after touch-ups, not after the first session. In the first few weeks, the color will go through several stages — it will fade, even out, and only then will it reveal its true beauty. I am here to guide you step by step, I will provide you with a personalized care guide, and if you follow all these instructions, your eyebrows will look flawless and enhance your face for a long time.</t>
+    <t>link raspuns</t>
+  </si>
+  <si>
+    <t>Defined smile through lips dermopigmentation</t>
+  </si>
+  <si>
+    <t>Discover how lip dermopigmentation can add depth and sensuality to your smile.</t>
+  </si>
+  <si>
+    <t>We have prepared the most important questions and answers about lip dermopigmentation, explained clearly, both in text and video, so that you know exactly what to expect from this procedure.</t>
+  </si>
+  <si>
+    <t>What is lips dermopigmentation?</t>
+  </si>
+  <si>
+    <t>A smile is one of the most beautiful expressions we wear, and the color and contour of the lips can give it more harmony and radiance. Lip dermopigmentation is a technique by which I delicately restore or intensify the natural shade of the lips, correct small asymmetries, and create a fine contour, so that they always look full of life.
+It is an ideal choice if your lips are very pale, have lost pigment over time, or if you want to even out the color or give them a fresher and more defined look without using lipstick every day.
+The procedure is performed using a professional dermograph and special pigments, chosen in shades that match your skin tone and complement your features. The final result can be very discreet, for a natural "my lips but better" effect, or more intense, depending on your wishes.
+Lip dermopigmentation does not mean a strong, rigid color, but a transparent, warm shade that blends perfectly with the texture of your lips. The pigment gradually fades over time, allowing you to adjust or refresh the color whenever you feel the need.
+The end result? Lips with a more defined contour, uniform color, and healthy appearance that will make your smile stand out in the most beautiful way, every day, effortlessly.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/5mVL5l7AcaQ</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -906,32 +930,7 @@
 Your safety and health always come first. Dermopigmentation is about beauty, but above all about care, responsibility, and respect for your body.</t>
   </si>
   <si>
-    <t>https://youtu.be/qpF18FTEhR0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-When it comes to lips, pigment is everything. This is an area with a higher pH, rich vascularization, and a natural shade that varies greatly from person to person, so color selection must be extremely careful and personalized.
-I use professional, biocompatible, and hypoallergenic cosmetic pigments, specially formulated to last on the lips without changing tone over time. These pigments are designed to preserve the beauty of the color and fade gradually and elegantly, so you can make adjustments when you want a refresh.
-When selecting the shade, I look at the tone and undertone of your skin: warm, cool, or neutral, the natural color of your lips, their natural pigmentation (more uniform or with paler areas), and the desired final effect: maybe you want a natural look, like your lips, but fresher, or maybe you want a more saturated color, inspired by your favorite lipstick.
-An important detail: in the case of lips with very cold or dark natural pigment (as sometimes happens due to genetic causes or after certain treatments), tone neutralization sessions may be necessary before applying the desired color. This ensures a uniform and beautiful result.
-In the end, the pigment we choose together is the perfect combination of safety, durability, and harmony with your natural beauty.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/wchI4eoAIe0</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134712943/777ba19052?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134711847/ca1efbf32c?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-This is a question I get asked very often, and it's natural for you to have it in mind too. The short answer is: because every skin is unique and reacts differently to pigment.
-After the first dermopigmentation session, the treated area, whether it's the eyebrows, lips, or areolas, looks more intense. The pigment is freshly deposited, and the skin is slightly inflamed. Over the next few weeks, during the natural healing process, the color begins to fade and settle until it reaches its final shade.
-During this period, the skin naturally eliminates a percentage of the pigment. This is the body's normal reaction to any element introduced from the outside. This is where the touch-up comes in: it is the second session in which we fill in the areas where the pigment has settled less, even out the color, adjust the symmetry if necessary, and strengthen the contours.
-Touch-ups are essential for a uniform, long-lasting, and natural-looking result. Once the skin has "gotten used" to the pigment during the first procedure, it will accept it much better during the second, which makes the final result stable and beautiful over time.
-In short: the first procedure prepares the ground, and the touch-up finishes the job. Without touch-ups, the result is only half complete. With touch-ups, you get the eyebrows, lips, or areolas you want, for longer and without surprises.</t>
+    <t>https://vimeo.com/1134711822/0140c6e130?fl=ls&amp;fe=ec</t>
   </si>
   <si>
     <t>What you need to do before eyeliner dermopigmentation?</t>
@@ -949,6 +948,35 @@
   </si>
   <si>
     <t>https://youtu.be/LPt0V9YqShM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+When it comes to lips, pigment is everything. This is an area with a higher pH, rich vascularization, and a natural shade that varies greatly from person to person, so color selection must be extremely careful and personalized.
+I use professional, biocompatible, and hypoallergenic cosmetic pigments, specially formulated to last on the lips without changing tone over time. These pigments are designed to preserve the beauty of the color and fade gradually and elegantly, so you can make adjustments when you want a refresh.
+When selecting the shade, I look at the tone and undertone of your skin: warm, cool, or neutral, the natural color of your lips, their natural pigmentation (more uniform or with paler areas), and the desired final effect: maybe you want a natural look, like your lips, but fresher, or maybe you want a more saturated color, inspired by your favorite lipstick.
+An important detail: in the case of lips with very cold or dark natural pigment (as sometimes happens due to genetic causes or after certain treatments), tone neutralization sessions may be necessary before applying the desired color. This ensures a uniform and beautiful result.
+In the end, the pigment we choose together is the perfect combination of safety, durability, and harmony with your natural beauty.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/wchI4eoAIe0</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134713994/80e9d0dc68?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134711847/ca1efbf32c?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>After getting eyeliner dermopigmentation, your eyes will need a little extra pampering and attention. It's nothing complicated, but every detail matters to ensure that the result remains beautiful, clear, and uniform for years to come.
+In the first few days, it is normal to feel a slight sensitivity, a feeling of "heavier" eyes, or even a slight swelling of the eyelids; this is just the way the skin reacts to the procedure. Apply cold compresses (not ice directly on the skin) for a few minutes, 2-3 times a day, to soothe the area.
+Very important: do not rub your eyes, pull on the skin of your eyelids, or try to remove any fine scabs that may form. Let them fall off on their own, otherwise you risk removing the pigment along with them.
+Throughout the healing period, avoid makeup around the eyes, mascara, liquid or cream eyeliner, and do not use oily makeup removers. Clean the area gently, using only water or special recommended solutions, and completely avoid swimming pools, saunas, or hot baths, as excessive heat and humidity can affect pigment fixation.
+Protect your eyes from strong sunlight. Wear large sunglasses with UV protection, even when it doesn't seem very bright outside, as UV radiation can degrade the pigment faster than you might think.
+In the first few weeks, avoid cosmetic treatments in the eye area: eyelash lifting, lamination, extensions, or laser procedures. All of these should be postponed until after complete healing.
+I will always be just a message away if you have any questions or if you feel you need to check the progress of the healing together. By following these simple recommendations, your eyeliner will set beautifully and remain intense and harmonious for as long as possible.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/K-DFcWvmFEg</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -964,35 +992,22 @@
 In short: it is not completely sensation-free, but it is a procedure designed to be gentle, safe, and bearable, so that your experience is as relaxed and stress-free as possible.</t>
   </si>
   <si>
-    <t>https://vimeo.com/1134713994/80e9d0dc68?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>The duration of the results varies, but in general, you can enjoy beautiful eyebrows for between 1 and 3 years. The difference depends on several factors: skin type, the shade of pigment chosen, lifestyle, and, above all, aftercare.
-In the first few weeks, the eyebrows go through a natural healing process: the color gradually lightens and settles evenly. To preserve the result for as long as possible, it is important to let the skin heal at its own pace, not to remove the scabs, and to protect the area from the sun by always using a high SPF.
-In the long term, there are factors that can accelerate pigment fading, such as products containing vitamin C, retinoids, or exfoliating acids, frequent exposure to chlorinated water, or tanning beds. Lighter shades, such as blonde or light brown, also tend to lose their intensity faster than darker ones.
-To maintain a clear shape and vibrant color, I recommend maintenance touch-ups whenever you feel your eyebrows need a refresh.
-Essentially, I lay the foundation for a lasting result, and you, through daily care, keep it beautiful for as long as possible.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/Lq8mWDiICOg</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134712991/2a713496a8?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>After getting eyeliner dermopigmentation, your eyes will need a little extra pampering and attention. It's nothing complicated, but every detail matters to ensure that the result remains beautiful, clear, and uniform for years to come.
-In the first few days, it is normal to feel a slight sensitivity, a feeling of "heavier" eyes, or even a slight swelling of the eyelids; this is just the way the skin reacts to the procedure. Apply cold compresses (not ice directly on the skin) for a few minutes, 2-3 times a day, to soothe the area.
-Very important: do not rub your eyes, pull on the skin of your eyelids, or try to remove any fine scabs that may form. Let them fall off on their own, otherwise you risk removing the pigment along with them.
-Throughout the healing period, avoid makeup around the eyes, mascara, liquid or cream eyeliner, and do not use oily makeup removers. Clean the area gently, using only water or special recommended solutions, and completely avoid swimming pools, saunas, or hot baths, as excessive heat and humidity can affect pigment fixation.
-Protect your eyes from strong sunlight. Wear large sunglasses with UV protection, even when it doesn't seem very bright outside, as UV radiation can degrade the pigment faster than you might think.
-In the first few weeks, avoid cosmetic treatments in the eye area: eyelash lifting, lamination, extensions, or laser procedures. All of these should be postponed until after complete healing.
-I will always be just a message away if you have any questions or if you feel you need to check the progress of the healing together. By following these simple recommendations, your eyeliner will set beautifully and remain intense and harmonious for as long as possible.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/K-DFcWvmFEg</t>
-  </si>
-  <si>
     <t>https://vimeo.com/1134711997/3982b6bf81?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>https://youtu.be/JuyJ4nI168U</t>
+  </si>
+  <si>
+    <t>https://vimeo.com/1134714942/5d895edf0f?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>Eyeliner obtained through dermopigmentation is one of the longest-lasting procedures, lasting on average between 2 and 4 years, sometimes even longer. This is due to both the delicate area we work on and the fact that the skin of the eyelids is protected from the sun, exfoliating products, and the daily friction to which other areas of the face are exposed.
+The fading process is much slower than with eyebrows. The pigment remains more stable and the line retains its clarity for longer. However, the exact duration depends on factors such as skin type, the intensity of the chosen color, individual metabolism, and the sensitivity of the skin around the eyes.
+Proper care immediately after the procedure plays an important role: avoiding makeup on the eyelids during the healing period, protecting the area from salt or chlorinated water, and following all hygiene recommendations will help the pigment to set optimally.
+Even though dermopigmented eyeliner lasts longer than other areas, maintenance touch-ups are recommended when you want to intensify the color again or adjust the shape, so you can enjoy perfectly contoured eyes for years to come.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/ucgOJ6tzIVY</t>
   </si>
   <si>
     <t>What you need to do before lips dermopigmentation?</t>
@@ -1011,22 +1026,10 @@
     <t>https://youtu.be/8iDUKg_dei0</t>
   </si>
   <si>
-    <t>https://youtu.be/JuyJ4nI168U</t>
+    <t>https://vimeo.com/1134714031/34d91ec018?fl=ls&amp;fe=ec</t>
   </si>
   <si>
     <t>https://vimeo.com/1134711831/6c523f503f?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134714942/5d895edf0f?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>Eyeliner obtained through dermopigmentation is one of the longest-lasting procedures, lasting on average between 2 and 4 years, sometimes even longer. This is due to both the delicate area we work on and the fact that the skin of the eyelids is protected from the sun, exfoliating products, and the daily friction to which other areas of the face are exposed.
-The fading process is much slower than with eyebrows. The pigment remains more stable and the line retains its clarity for longer. However, the exact duration depends on factors such as skin type, the intensity of the chosen color, individual metabolism, and the sensitivity of the skin around the eyes.
-Proper care immediately after the procedure plays an important role: avoiding makeup on the eyelids during the healing period, protecting the area from salt or chlorinated water, and following all hygiene recommendations will help the pigment to set optimally.
-Even though dermopigmented eyeliner lasts longer than other areas, maintenance touch-ups are recommended when you want to intensify the color again or adjust the shape, so you can enjoy perfectly contoured eyes for years to come.</t>
-  </si>
-  <si>
-    <t>https://youtu.be/ucgOJ6tzIVY</t>
   </si>
   <si>
     <t>After getting lip micropigmentation, the healing period begins, which is just as important as the procedure itself in order to achieve a beautiful and even result.
@@ -1042,10 +1045,13 @@
     <t>https://youtu.be/mvw6P-rRa0I</t>
   </si>
   <si>
-    <t>https://vimeo.com/1134714031/34d91ec018?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
     <t>https://vimeo.com/1134711813/3c65d2ade5?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
+    <t>link YT</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Wtq40uMGhUo</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -1058,15 +1064,12 @@
     <t>https://youtu.be/SVCiTSEpoMc</t>
   </si>
   <si>
+    <t>https://vimeo.com/1134714931/b8760b6993?fl=ls&amp;fe=ec</t>
+  </si>
+  <si>
     <t>https://vimeo.com/1134711857/0612346b14?fl=ls&amp;fe=ec</t>
   </si>
   <si>
-    <t>link YT</t>
-  </si>
-  <si>
-    <t>https://youtu.be/Wtq40uMGhUo</t>
-  </si>
-  <si>
     <t>pregatire: https://youtu.be/8pFARdC9wvI</t>
   </si>
   <si>
@@ -1083,9 +1086,6 @@
   </si>
   <si>
     <t>pregatire: https://vimeo.com/1134711988/44f0ef4fde?fl=ls&amp;fe=ec</t>
-  </si>
-  <si>
-    <t>https://vimeo.com/1134714931/b8760b6993?fl=ls&amp;fe=ec</t>
   </si>
   <si>
     <t>intretinere: https://vimeo.com/1134711974/036ab09005?fl=ls&amp;fe=ec</t>
@@ -1112,13 +1112,13 @@
       <color rgb="FF0000FF"/>
     </font>
     <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
+    <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0000FF"/>
     </font>
     <font>
       <u/>
@@ -1194,16 +1194,16 @@
     <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1468,227 +1468,227 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>82</v>
+        <v>104</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>91</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="D8" s="11"/>
+        <v>112</v>
+      </c>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="D8" s="12"/>
       <c r="E8" s="1" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="1" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="1" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="1" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="1" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="1" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="1" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -1721,32 +1721,32 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D1" s="1"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="6">
@@ -1773,20 +1773,20 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C1" s="1"/>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2">
@@ -1794,132 +1794,132 @@
         <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C2" s="1"/>
       <c r="H2" s="2" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>34</v>
-      </c>
       <c r="F4" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="I4" s="3"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>58</v>
+        <v>50</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="F6" s="6" t="s">
         <v>54</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>107</v>
+        <v>100</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>130</v>
+        <v>108</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>135</v>
+        <v>78</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>136</v>
+        <v>86</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>147</v>
+      <c r="A13" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>94</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
@@ -1933,7 +1933,7 @@
       <c r="L13" s="13"/>
     </row>
     <row r="14">
-      <c r="A14" s="12"/>
+      <c r="A14" s="11"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
@@ -2241,10 +2241,10 @@
       <c r="L44" s="13"/>
     </row>
     <row r="100">
-      <c r="A100" s="12" t="s">
+      <c r="A100" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="B100" s="12" t="s">
+      <c r="B100" s="11" t="s">
         <v>149</v>
       </c>
       <c r="C100" s="13"/>
@@ -2254,13 +2254,13 @@
     </row>
     <row r="101">
       <c r="A101" s="13"/>
-      <c r="B101" s="12" t="s">
+      <c r="B101" s="11" t="s">
         <v>150</v>
       </c>
       <c r="C101" s="13"/>
       <c r="D101" s="13"/>
       <c r="E101" s="13"/>
-      <c r="F101" s="12" t="s">
+      <c r="F101" s="11" t="s">
         <v>151</v>
       </c>
     </row>
@@ -2274,110 +2274,110 @@
     </row>
     <row r="103">
       <c r="A103" s="13"/>
-      <c r="B103" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="C103" s="12" t="s">
+      <c r="B103" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="D103" s="12" t="s">
+      <c r="C103" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="E103" s="12" t="s">
+      <c r="D103" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="F103" s="12" t="s">
+      <c r="E103" s="11" t="s">
         <v>156</v>
+      </c>
+      <c r="F103" s="11" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="13"/>
-      <c r="B104" s="12" t="s">
-        <v>157</v>
+      <c r="B104" s="11" t="s">
+        <v>159</v>
       </c>
       <c r="C104" s="13"/>
       <c r="D104" s="13"/>
       <c r="E104" s="13"/>
-      <c r="F104" s="12" t="s">
-        <v>156</v>
+      <c r="F104" s="11" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="13"/>
-      <c r="B105" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="C105" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="D105" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="E105" s="12" t="s">
-        <v>160</v>
+      <c r="B105" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C105" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="D105" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="E105" s="11" t="s">
+        <v>164</v>
       </c>
       <c r="F105" s="13"/>
     </row>
     <row r="106">
       <c r="A106" s="13"/>
       <c r="B106" s="14" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C106" s="13"/>
-      <c r="D106" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="E106" s="12" t="s">
-        <v>163</v>
+      <c r="D106" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="E106" s="11" t="s">
+        <v>169</v>
       </c>
       <c r="F106" s="13"/>
     </row>
     <row r="107">
       <c r="A107" s="13"/>
-      <c r="B107" s="12" t="s">
-        <v>164</v>
+      <c r="B107" s="11" t="s">
+        <v>170</v>
       </c>
       <c r="C107" s="13"/>
       <c r="D107" s="13"/>
       <c r="E107" s="13"/>
-      <c r="F107" s="12" t="s">
-        <v>166</v>
+      <c r="F107" s="11" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="13"/>
-      <c r="B108" s="12" t="s">
-        <v>168</v>
+      <c r="B108" s="11" t="s">
+        <v>172</v>
       </c>
       <c r="C108" s="13"/>
       <c r="D108" s="13"/>
       <c r="E108" s="13"/>
-      <c r="F108" s="12" t="s">
-        <v>169</v>
+      <c r="F108" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="13"/>
-      <c r="B109" s="12" t="s">
-        <v>172</v>
+      <c r="B109" s="11" t="s">
+        <v>174</v>
       </c>
       <c r="C109" s="13"/>
       <c r="D109" s="13"/>
       <c r="E109" s="13"/>
-      <c r="F109" s="12" t="s">
-        <v>169</v>
+      <c r="F109" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="13"/>
       <c r="B110" s="14" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C110" s="13"/>
       <c r="D110" s="13"/>
       <c r="E110" s="13"/>
-      <c r="F110" s="12" t="s">
-        <v>169</v>
+      <c r="F110" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="111">
@@ -2388,8 +2388,8 @@
       <c r="C111" s="13"/>
       <c r="D111" s="13"/>
       <c r="E111" s="13"/>
-      <c r="F111" s="12" t="s">
-        <v>169</v>
+      <c r="F111" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="112">
@@ -2400,82 +2400,82 @@
       <c r="C112" s="13"/>
       <c r="D112" s="13"/>
       <c r="E112" s="13"/>
-      <c r="F112" s="12" t="s">
-        <v>169</v>
+      <c r="F112" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="13"/>
-      <c r="B113" s="12" t="s">
-        <v>178</v>
+      <c r="B113" s="11" t="s">
+        <v>179</v>
       </c>
       <c r="C113" s="13"/>
       <c r="D113" s="13"/>
       <c r="E113" s="13"/>
-      <c r="F113" s="12" t="s">
-        <v>169</v>
+      <c r="F113" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="13"/>
       <c r="B114" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="C114" s="12" t="s">
         <v>180</v>
+      </c>
+      <c r="C114" s="11" t="s">
+        <v>181</v>
       </c>
       <c r="D114" s="13"/>
       <c r="E114" s="13"/>
-      <c r="F114" s="12" t="s">
-        <v>169</v>
+      <c r="F114" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="13"/>
-      <c r="B115" s="12" t="s">
-        <v>181</v>
+      <c r="B115" s="11" t="s">
+        <v>182</v>
       </c>
       <c r="C115" s="13"/>
       <c r="D115" s="13"/>
       <c r="E115" s="13"/>
-      <c r="F115" s="12" t="s">
-        <v>169</v>
+      <c r="F115" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="13"/>
-      <c r="B116" s="12" t="s">
-        <v>182</v>
+      <c r="B116" s="11" t="s">
+        <v>183</v>
       </c>
       <c r="C116" s="13"/>
       <c r="D116" s="13"/>
       <c r="E116" s="13"/>
-      <c r="F116" s="12" t="s">
-        <v>169</v>
+      <c r="F116" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="13"/>
-      <c r="B117" s="12" t="s">
-        <v>183</v>
+      <c r="B117" s="11" t="s">
+        <v>184</v>
       </c>
       <c r="C117" s="13"/>
       <c r="D117" s="13"/>
       <c r="E117" s="13"/>
-      <c r="F117" s="12" t="s">
-        <v>169</v>
+      <c r="F117" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="13"/>
-      <c r="B118" s="12" t="s">
-        <v>184</v>
+      <c r="B118" s="11" t="s">
+        <v>186</v>
       </c>
       <c r="C118" s="13"/>
       <c r="D118" s="13"/>
       <c r="E118" s="13"/>
-      <c r="F118" s="12" t="s">
-        <v>169</v>
+      <c r="F118" s="11" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="119">
@@ -2488,8 +2488,8 @@
     </row>
     <row r="120">
       <c r="A120" s="13"/>
-      <c r="B120" s="12" t="s">
-        <v>186</v>
+      <c r="B120" s="11" t="s">
+        <v>188</v>
       </c>
       <c r="C120" s="13"/>
       <c r="D120" s="13"/>
@@ -2529,16 +2529,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
@@ -2546,141 +2546,141 @@
         <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>50</v>
+        <v>39</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="G6" s="6" t="s">
         <v>54</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B8" s="9"/>
       <c r="C8" s="8" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="9"/>
       <c r="F8" s="10" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="H8" s="9"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>99</v>
+        <v>72</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>119</v>
+        <v>73</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>74</v>
       </c>
       <c r="H9" s="3"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>134</v>
+        <v>76</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>135</v>
+        <v>78</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>136</v>
+        <v>86</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>141</v>
+        <v>87</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>145</v>
+        <v>88</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>90</v>
       </c>
       <c r="H11" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>147</v>
+      <c r="A14" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2715,16 +2715,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
@@ -2732,135 +2732,135 @@
         <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="G6" s="6" t="s">
         <v>54</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>89</v>
+        <v>98</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>112</v>
+        <v>109</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>135</v>
+        <v>78</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>136</v>
+        <v>86</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>147</v>
+      <c r="A13" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2898,21 +2898,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="1" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3">
@@ -2920,48 +2920,48 @@
         <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="6" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>191</v>
@@ -2969,103 +2969,103 @@
       <c r="F7" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="6" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>61</v>
+      <c r="G8" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>71</v>
+        <v>60</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>214</v>
+        <v>196</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>219</v>
+        <v>198</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>222</v>
+        <v>202</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>204</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>225</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>227</v>
+        <v>211</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>135</v>
+        <v>78</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>136</v>
+        <v>86</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>233</v>
+        <v>214</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>235</v>
+        <v>215</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="15">
       <c r="F15" s="1"/>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>147</v>
+      <c r="A16" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -3109,21 +3109,21 @@
     <row r="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3">
@@ -3131,71 +3131,71 @@
         <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>201</v>
+        <v>208</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>61</v>
+      <c r="G7" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>71</v>
+        <v>60</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="9">
@@ -3209,18 +3209,18 @@
         <v>230</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>236</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>237</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>238</v>
@@ -3228,38 +3228,38 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>227</v>
+        <v>211</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>135</v>
+        <v>78</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>136</v>
+        <v>86</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="F12" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="G12" s="7" t="s">
-        <v>249</v>
-      </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>147</v>
+      <c r="A14" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -3298,21 +3298,21 @@
     <row r="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3">
@@ -3320,135 +3320,135 @@
         <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>226</v>
+        <v>232</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>61</v>
+      <c r="G7" s="6" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>71</v>
+        <v>60</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>243</v>
+        <v>244</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="G10" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="G10" s="6" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>227</v>
+        <v>211</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>135</v>
+        <v>78</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>136</v>
+        <v>86</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>147</v>
+      <c r="A14" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="15">
@@ -3489,15 +3489,15 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>244</v>
+        <v>239</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -3519,18 +3519,18 @@
     <row r="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>255</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="3">

</xml_diff>